<commit_message>
Update VDS analysis (sectors only).xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/VDS analysis (sectors only).xlsx
+++ b/clustering/sepsectors/VDS analysis (sectors only).xlsx
@@ -9,18 +9,19 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12885"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12885" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="sectors" sheetId="1" r:id="rId1"/>
     <sheet name="patterns" sheetId="2" r:id="rId2"/>
+    <sheet name="Лист1" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="38">
   <si>
     <t>sector</t>
   </si>
@@ -140,6 +141,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -189,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -200,6 +204,23 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -215,6 +236,977 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="ru-RU"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Лист1!$D$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>VDS_s</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Лист1!$C$11:$C$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2021</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2022</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2024</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Лист1!$D$11:$D$15</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0.90005264112546035</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.89505619534025793</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.80665071075171224</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.7526672034694295</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1910-400C-B1D7-3A0C47776EF4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Лист1!$E$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>skvozcosts_s</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Лист1!$C$11:$C$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2021</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2022</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2024</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Лист1!$E$11:$E$15</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0.99712272572842708</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.33436699801812092</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.71526368042226229</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.1091276476172726</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-1910-400C-B1D7-3A0C47776EF4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1185930784"/>
+        <c:axId val="1185932864"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1185930784"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1185932864"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1185932864"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1185930784"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="ru-RU"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="ru-RU"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>409574</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>66674</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>42863</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Диаграмма 2"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3489,4 +4481,260 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A3:H19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="76.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2020</v>
+      </c>
+      <c r="D4" s="2">
+        <v>3790890.0205506901</v>
+      </c>
+      <c r="E4" s="3">
+        <v>56.713594025000013</v>
+      </c>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D5" s="2">
+        <v>4211853.6709257532</v>
+      </c>
+      <c r="E5" s="3">
+        <v>56.877245459999997</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0.11</v>
+      </c>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D6" s="2">
+        <v>3769845.722028703</v>
+      </c>
+      <c r="E6" s="3">
+        <v>19.017873819999998</v>
+      </c>
+      <c r="F6" s="8">
+        <v>-0.11</v>
+      </c>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D7" s="2">
+        <v>3397494.7572344672</v>
+      </c>
+      <c r="E7" s="3">
+        <v>40.68222792000001</v>
+      </c>
+      <c r="F7" s="8">
+        <v>-0.1</v>
+      </c>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D8" s="2">
+        <v>3170124.123918138</v>
+      </c>
+      <c r="E8" s="3">
+        <v>6.2068799999999991</v>
+      </c>
+      <c r="F8" s="9">
+        <v>-6.6000000000000003E-2</v>
+      </c>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2020</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0.90005264112546035</v>
+      </c>
+      <c r="E11" s="4">
+        <v>0.99712272572842708</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0.89505619534025793</v>
+      </c>
+      <c r="E13" s="4">
+        <v>0.33436699801812092</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0.80665071075171224</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0.71526368042226229</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.7526672034694295</v>
+      </c>
+      <c r="E15" s="4">
+        <v>0.1091276476172726</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E19" s="10"/>
+    </row>
+  </sheetData>
+  <sortState ref="C11:E15">
+    <sortCondition ref="C11:C15"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>